<commit_message>
Added detailed pc setup information
git-svn-id: http://10.105.1.46/svn/CCRT/Ccrt/branches/Common3700@18805 80089e14-fa6c-c64e-badd-1f0333e23b03
</commit_message>
<xml_diff>
--- a/Source/Isuzu/Isuzu Plant Matrix.xlsx
+++ b/Source/Isuzu/Isuzu Plant Matrix.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="78">
   <si>
     <t>6.2.1</t>
   </si>
@@ -147,12 +147,6 @@
     <t>baud rate 15765</t>
   </si>
   <si>
-    <t>Persistant data such as logs / cal files / build data is stored in C:\FlashStation\</t>
-  </si>
-  <si>
-    <t>Specification of input device and vehicle comm device stored in C:\Users\USERNAME\AppData\Local\Burke_E._Porter\</t>
-  </si>
-  <si>
     <t>Bom</t>
   </si>
   <si>
@@ -165,7 +159,97 @@
     <t>To install, remove program through control panel, then run setup.exe from setup project</t>
   </si>
   <si>
-    <t>Program settings stored in C:\Users\USERNAME\AppData\Local\Burke_E._Porter\</t>
+    <t>Windows 7</t>
+  </si>
+  <si>
+    <t>Isuzu_Charlotte</t>
+  </si>
+  <si>
+    <t>192.168.1.1</t>
+  </si>
+  <si>
+    <t>10.50.2.2</t>
+  </si>
+  <si>
+    <t>192.168.1.2</t>
+  </si>
+  <si>
+    <t>255.255.255.1</t>
+  </si>
+  <si>
+    <t>10.50.2.1</t>
+  </si>
+  <si>
+    <t>255.255.0.0</t>
+  </si>
+  <si>
+    <t>10.50.1.254</t>
+  </si>
+  <si>
+    <t>dns: 10.1.1.27</t>
+  </si>
+  <si>
+    <t>dns: 10.1.1.28</t>
+  </si>
+  <si>
+    <t>GUI Computer Name</t>
+  </si>
+  <si>
+    <t>CCRT</t>
+  </si>
+  <si>
+    <t>login: Spartan pass: spartan</t>
+  </si>
+  <si>
+    <t>IsuzuMemory</t>
+  </si>
+  <si>
+    <t>(wireless)</t>
+  </si>
+  <si>
+    <t>192.168.1.99</t>
+  </si>
+  <si>
+    <t>192.168.1.100</t>
+  </si>
+  <si>
+    <t>G drive mapped to 192.168.1.3\home\CCRT</t>
+  </si>
+  <si>
+    <t>Additional users</t>
+  </si>
+  <si>
+    <t xml:space="preserve">network id: Isuzu_EOL pass:bepIsuzu </t>
+  </si>
+  <si>
+    <t>login: DVT_Transfer pass: Q48s^PT1</t>
+  </si>
+  <si>
+    <t>C:\Bom folder shared to these users</t>
+  </si>
+  <si>
+    <t>sl7804 card dip settings</t>
+  </si>
+  <si>
+    <t>1 off 2 - 7 on</t>
+  </si>
+  <si>
+    <t>Wireless router used for connection to Flash Station</t>
+  </si>
+  <si>
+    <t>Bom processor receives build of materials in shared folder and processes into vehilce build records</t>
+  </si>
+  <si>
+    <t>These are placed in the configuration build records directory on the qnx pc - flash station monitors this folder for these files and transfers locally</t>
+  </si>
+  <si>
+    <t>Result files are placed in a shared forlder for the plant system to retreive</t>
+  </si>
+  <si>
+    <t>ESN is placed in a shared folder by plant system - this is used by the flash station to write to the Engine controller and by the rolls pc to verify</t>
+  </si>
+  <si>
+    <t>Persistant data such as logs / cal files / build data /esn are stored in C:\FlashStation\</t>
   </si>
 </sst>
 </file>
@@ -419,7 +503,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -505,6 +589,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -810,7 +897,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O70"/>
+  <dimension ref="A1:P68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.28515625" bestFit="1" customWidth="1"/>
@@ -819,16 +906,18 @@
     <col min="5" max="5" width="30.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.42578125" customWidth="1"/>
-    <col min="12" max="12" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="32.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.42578125" customWidth="1"/>
+    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -905,22 +994,32 @@
       <c r="F9" s="28"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F10" s="18"/>
+      <c r="B10" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F11" s="18"/>
+      <c r="B11" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F12" s="18"/>
+      <c r="B12" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F13" s="18"/>
+      <c r="B13" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F14" s="18"/>
+      <c r="B14" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F15" s="18"/>
+      <c r="F15" s="19"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
@@ -928,10 +1027,10 @@
       </c>
       <c r="F16" s="19"/>
     </row>
-    <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
     </row>
-    <row r="18" spans="1:15" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="20" t="s">
         <v>15</v>
       </c>
@@ -960,89 +1059,125 @@
         <v>26</v>
       </c>
       <c r="J18" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="K18" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="K18" s="23" t="s">
+      <c r="L18" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="L18" s="23" t="s">
+      <c r="M18" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="M18" s="23" t="s">
+      <c r="N18" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="N18" s="22" t="s">
+      <c r="O18" s="22" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="17">
         <v>1</v>
       </c>
-      <c r="B19" s="31"/>
+      <c r="B19" s="31">
+        <v>507382</v>
+      </c>
       <c r="C19" s="31">
         <v>3600</v>
       </c>
-      <c r="D19" s="5"/>
+      <c r="D19" s="5" t="s">
+        <v>47</v>
+      </c>
       <c r="E19" s="5" t="s">
         <v>0</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
+      <c r="G19" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="J19" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="K19" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="K19" s="5" t="s">
+      <c r="L19" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="L19" s="5">
+      <c r="M19" s="5">
         <v>507382</v>
       </c>
-      <c r="M19" s="5"/>
-      <c r="N19" s="18"/>
-      <c r="O19" s="24"/>
-    </row>
-    <row r="20" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N19" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="O19" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="P19" s="24"/>
+    </row>
+    <row r="20" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
+      <c r="E20" s="5" t="s">
+        <v>70</v>
+      </c>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
+      <c r="H20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>66</v>
+      </c>
       <c r="K20" s="5"/>
       <c r="L20" s="5"/>
       <c r="M20" s="5"/>
-      <c r="N20" s="18"/>
-      <c r="O20" s="24"/>
-    </row>
-    <row r="21" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="14" t="s">
-        <v>35</v>
-      </c>
+      <c r="N20" s="5"/>
+      <c r="O20" s="18"/>
+      <c r="P20" s="24"/>
+    </row>
+    <row r="21" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="14"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
+      <c r="E21" s="5" t="s">
+        <v>71</v>
+      </c>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
+      <c r="H21" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>60</v>
+      </c>
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
       <c r="M21" s="5"/>
-      <c r="N21" s="18"/>
-      <c r="O21" s="24"/>
-    </row>
-    <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N21" s="5"/>
+      <c r="O21" s="18"/>
+      <c r="P21" s="24"/>
+    </row>
+    <row r="22" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1051,15 +1186,20 @@
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
       <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
+      <c r="I22" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J22" s="37" t="s">
+        <v>68</v>
+      </c>
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
-      <c r="N22" s="18"/>
-      <c r="O22" s="24"/>
-    </row>
-    <row r="23" spans="1:15" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N22" s="5"/>
+      <c r="O22" s="18"/>
+      <c r="P22" s="24"/>
+    </row>
+    <row r="23" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="15"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1068,15 +1208,20 @@
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
       <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
+      <c r="I23" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>69</v>
+      </c>
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
       <c r="M23" s="5"/>
-      <c r="N23" s="18"/>
-      <c r="O23" s="24"/>
-    </row>
-    <row r="24" spans="1:15" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N23" s="5"/>
+      <c r="O23" s="18"/>
+      <c r="P23" s="24"/>
+    </row>
+    <row r="24" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="17"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1086,14 +1231,17 @@
       <c r="G24" s="5"/>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
+      <c r="J24" s="5" t="s">
+        <v>65</v>
+      </c>
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
       <c r="M24" s="5"/>
-      <c r="N24" s="18"/>
-      <c r="O24" s="24"/>
-    </row>
-    <row r="25" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N24" s="5"/>
+      <c r="O24" s="18"/>
+      <c r="P24" s="24"/>
+    </row>
+    <row r="25" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="17"/>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
@@ -1107,27 +1255,37 @@
       <c r="K25" s="5"/>
       <c r="L25" s="5"/>
       <c r="M25" s="5"/>
-      <c r="N25" s="18"/>
-      <c r="O25" s="24"/>
-    </row>
-    <row r="26" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="17"/>
+      <c r="N25" s="5"/>
+      <c r="O25" s="18"/>
+      <c r="P25" s="24"/>
+    </row>
+    <row r="26" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="17" t="s">
+        <v>35</v>
+      </c>
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
+      <c r="D26" s="11" t="s">
+        <v>47</v>
+      </c>
       <c r="E26" s="5"/>
       <c r="F26" s="5"/>
       <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
+      <c r="H26" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
+      <c r="J26" s="5" t="s">
+        <v>61</v>
+      </c>
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
       <c r="M26" s="5"/>
-      <c r="N26" s="18"/>
-      <c r="O26" s="24"/>
-    </row>
-    <row r="27" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N26" s="5"/>
+      <c r="O26" s="18"/>
+      <c r="P26" s="24"/>
+    </row>
+    <row r="27" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="17"/>
       <c r="B27" s="11"/>
       <c r="C27" s="11"/>
@@ -1135,16 +1293,19 @@
       <c r="E27" s="5"/>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
+      <c r="H27" s="5" t="s">
+        <v>54</v>
+      </c>
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
       <c r="K27" s="5"/>
       <c r="L27" s="5"/>
       <c r="M27" s="5"/>
-      <c r="N27" s="18"/>
-      <c r="O27" s="24"/>
-    </row>
-    <row r="28" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N27" s="5"/>
+      <c r="O27" s="18"/>
+      <c r="P27" s="24"/>
+    </row>
+    <row r="28" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="14"/>
       <c r="B28" s="11"/>
       <c r="C28" s="11"/>
@@ -1152,16 +1313,19 @@
       <c r="E28" s="5"/>
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
+      <c r="H28" s="5" t="s">
+        <v>64</v>
+      </c>
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
       <c r="K28" s="5"/>
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
-      <c r="N28" s="18"/>
-      <c r="O28" s="24"/>
-    </row>
-    <row r="29" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N28" s="5"/>
+      <c r="O28" s="18"/>
+      <c r="P28" s="24"/>
+    </row>
+    <row r="29" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="14"/>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -1169,16 +1333,19 @@
       <c r="E29" s="5"/>
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
+      <c r="H29" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
       <c r="K29" s="5"/>
       <c r="L29" s="5"/>
       <c r="M29" s="5"/>
-      <c r="N29" s="18"/>
-      <c r="O29" s="24"/>
-    </row>
-    <row r="30" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N29" s="5"/>
+      <c r="O29" s="18"/>
+      <c r="P29" s="24"/>
+    </row>
+    <row r="30" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="16"/>
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
@@ -1186,16 +1353,19 @@
       <c r="E30" s="5"/>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
+      <c r="H30" s="5" t="s">
+        <v>67</v>
+      </c>
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
       <c r="K30" s="5"/>
       <c r="L30" s="5"/>
       <c r="M30" s="5"/>
-      <c r="N30" s="18"/>
-      <c r="O30" s="24"/>
-    </row>
-    <row r="31" spans="1:15" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N30" s="5"/>
+      <c r="O30" s="18"/>
+      <c r="P30" s="24"/>
+    </row>
+    <row r="31" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="15"/>
       <c r="B31" s="32"/>
       <c r="C31" s="32"/>
@@ -1209,10 +1379,11 @@
       <c r="K31" s="5"/>
       <c r="L31" s="5"/>
       <c r="M31" s="5"/>
-      <c r="N31" s="18"/>
-      <c r="O31" s="24"/>
-    </row>
-    <row r="32" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="N31" s="5"/>
+      <c r="O31" s="18"/>
+      <c r="P31" s="24"/>
+    </row>
+    <row r="32" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B32" s="25"/>
       <c r="C32" s="25"/>
       <c r="D32" s="28"/>
@@ -1221,19 +1392,20 @@
       <c r="G32" s="25"/>
       <c r="H32" s="25"/>
       <c r="I32" s="28"/>
-      <c r="J32" s="25"/>
+      <c r="J32" s="28"/>
       <c r="K32" s="25"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="25"/>
+      <c r="L32" s="25"/>
+      <c r="M32" s="28"/>
       <c r="N32" s="25"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="O32" s="25"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="37" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="37" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>14</v>
       </c>
@@ -1251,10 +1423,11 @@
       <c r="G37" s="27"/>
       <c r="H37" s="27"/>
       <c r="I37" s="27"/>
-      <c r="J37" s="22"/>
-      <c r="K37" s="21"/>
-    </row>
-    <row r="38" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J37" s="27"/>
+      <c r="K37" s="22"/>
+      <c r="L37" s="21"/>
+    </row>
+    <row r="38" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="17" t="s">
         <v>18</v>
       </c>
@@ -1266,10 +1439,11 @@
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
-      <c r="J38" s="28"/>
-      <c r="K38" s="24"/>
-    </row>
-    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J38" s="2"/>
+      <c r="K38" s="28"/>
+      <c r="L38" s="24"/>
+    </row>
+    <row r="39" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="36" t="s">
         <v>20</v>
       </c>
@@ -1280,10 +1454,11 @@
       <c r="G39" s="19"/>
       <c r="H39" s="19"/>
       <c r="I39" s="19"/>
-      <c r="J39" s="18"/>
-      <c r="K39" s="24"/>
-    </row>
-    <row r="40" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J39" s="19"/>
+      <c r="K39" s="18"/>
+      <c r="L39" s="24"/>
+    </row>
+    <row r="40" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="36" t="s">
         <v>19</v>
       </c>
@@ -1295,10 +1470,11 @@
       <c r="G40" s="19"/>
       <c r="H40" s="19"/>
       <c r="I40" s="19"/>
-      <c r="J40" s="18"/>
-      <c r="K40" s="24"/>
-    </row>
-    <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J40" s="19"/>
+      <c r="K40" s="18"/>
+      <c r="L40" s="24"/>
+    </row>
+    <row r="41" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="16" t="s">
         <v>13</v>
       </c>
@@ -1310,10 +1486,11 @@
       <c r="G41" s="19"/>
       <c r="H41" s="19"/>
       <c r="I41" s="19"/>
-      <c r="J41" s="18"/>
-      <c r="K41" s="24"/>
-    </row>
-    <row r="42" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J41" s="19"/>
+      <c r="K41" s="18"/>
+      <c r="L41" s="24"/>
+    </row>
+    <row r="42" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="16"/>
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
@@ -1323,10 +1500,11 @@
       <c r="G42" s="19"/>
       <c r="H42" s="19"/>
       <c r="I42" s="19"/>
-      <c r="J42" s="18"/>
-      <c r="K42" s="24"/>
-    </row>
-    <row r="43" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J42" s="19"/>
+      <c r="K42" s="18"/>
+      <c r="L42" s="24"/>
+    </row>
+    <row r="43" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="15"/>
       <c r="B43" s="2"/>
       <c r="D43" s="19"/>
@@ -1335,10 +1513,11 @@
       <c r="G43" s="19"/>
       <c r="H43" s="19"/>
       <c r="I43" s="19"/>
-      <c r="J43" s="18"/>
-      <c r="K43" s="24"/>
-    </row>
-    <row r="44" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J43" s="19"/>
+      <c r="K43" s="18"/>
+      <c r="L43" s="24"/>
+    </row>
+    <row r="44" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="15"/>
       <c r="B44" s="2"/>
       <c r="D44" s="19"/>
@@ -1347,10 +1526,11 @@
       <c r="G44" s="19"/>
       <c r="H44" s="19"/>
       <c r="I44" s="19"/>
-      <c r="J44" s="18"/>
-      <c r="K44" s="24"/>
-    </row>
-    <row r="45" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J44" s="19"/>
+      <c r="K44" s="18"/>
+      <c r="L44" s="24"/>
+    </row>
+    <row r="45" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="15"/>
       <c r="B45" s="2"/>
       <c r="D45" s="19"/>
@@ -1359,10 +1539,11 @@
       <c r="G45" s="19"/>
       <c r="H45" s="19"/>
       <c r="I45" s="19"/>
-      <c r="J45" s="18"/>
-      <c r="K45" s="24"/>
-    </row>
-    <row r="46" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J45" s="19"/>
+      <c r="K45" s="18"/>
+      <c r="L45" s="24"/>
+    </row>
+    <row r="46" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="15"/>
       <c r="B46" s="2"/>
       <c r="D46" s="19"/>
@@ -1371,10 +1552,11 @@
       <c r="G46" s="19"/>
       <c r="H46" s="19"/>
       <c r="I46" s="19"/>
-      <c r="J46" s="18"/>
-      <c r="K46" s="24"/>
-    </row>
-    <row r="47" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J46" s="19"/>
+      <c r="K46" s="18"/>
+      <c r="L46" s="24"/>
+    </row>
+    <row r="47" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="15"/>
       <c r="B47" s="2"/>
       <c r="D47" s="19"/>
@@ -1383,10 +1565,11 @@
       <c r="G47" s="19"/>
       <c r="H47" s="19"/>
       <c r="I47" s="19"/>
-      <c r="J47" s="18"/>
-      <c r="K47" s="24"/>
-    </row>
-    <row r="48" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J47" s="19"/>
+      <c r="K47" s="18"/>
+      <c r="L47" s="24"/>
+    </row>
+    <row r="48" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="15"/>
       <c r="B48" s="2"/>
       <c r="D48" s="19"/>
@@ -1395,10 +1578,11 @@
       <c r="G48" s="19"/>
       <c r="H48" s="19"/>
       <c r="I48" s="19"/>
-      <c r="J48" s="18"/>
-      <c r="K48" s="24"/>
-    </row>
-    <row r="49" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J48" s="19"/>
+      <c r="K48" s="18"/>
+      <c r="L48" s="24"/>
+    </row>
+    <row r="49" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="15"/>
       <c r="B49" s="2"/>
       <c r="D49" s="19"/>
@@ -1407,10 +1591,11 @@
       <c r="G49" s="19"/>
       <c r="H49" s="19"/>
       <c r="I49" s="19"/>
-      <c r="J49" s="18"/>
-      <c r="K49" s="24"/>
-    </row>
-    <row r="50" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J49" s="19"/>
+      <c r="K49" s="18"/>
+      <c r="L49" s="24"/>
+    </row>
+    <row r="50" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="15"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -1420,24 +1605,26 @@
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
-      <c r="J50" s="33"/>
-      <c r="K50" s="24"/>
-    </row>
-    <row r="51" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="J50" s="2"/>
+      <c r="K50" s="33"/>
+      <c r="L50" s="24"/>
+    </row>
+    <row r="51" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="D51" s="25"/>
       <c r="E51" s="25"/>
       <c r="F51" s="28"/>
       <c r="G51" s="25"/>
       <c r="H51" s="25"/>
       <c r="I51" s="28"/>
-      <c r="J51" s="25"/>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J51" s="28"/>
+      <c r="K51" s="25"/>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>35</v>
       </c>
@@ -1448,10 +1635,10 @@
         <v>39</v>
       </c>
       <c r="E56" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B57">
         <v>9600</v>
       </c>
@@ -1459,10 +1646,10 @@
         <v>41</v>
       </c>
       <c r="E57" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B58">
         <v>8</v>
       </c>
@@ -1470,7 +1657,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
         <v>37</v>
       </c>
@@ -1478,41 +1665,32 @@
         <v>42</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B60">
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B65" t="s">
-        <v>44</v>
+        <v>77</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B68" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B70" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Updated software to log reason for directory open failure. Added secondary attempt to retry ESN extraction from file.
git-svn-id: http://10.105.1.46/svn/CCRT/Ccrt/branches/Common3700@20448 80089e14-fa6c-c64e-badd-1f0333e23b03
</commit_message>
<xml_diff>
--- a/Source/Isuzu/Isuzu Plant Matrix.xlsx
+++ b/Source/Isuzu/Isuzu Plant Matrix.xlsx
@@ -16,10 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="96">
-  <si>
-    <t>6.2.1</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="95">
   <si>
     <t>S / N</t>
   </si>
@@ -114,9 +111,6 @@
     <t>Charlotte, MI</t>
   </si>
   <si>
-    <t>192.168.1.3</t>
-  </si>
-  <si>
     <t>Isuzu</t>
   </si>
   <si>
@@ -304,6 +298,9 @@
   </si>
   <si>
     <t>Qnx PC requires ccrtfp user in group 100</t>
+  </si>
+  <si>
+    <t>6.3.2</t>
   </si>
 </sst>
 </file>
@@ -321,6 +318,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -615,7 +613,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -720,6 +718,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1049,30 +1050,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="26" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="27" t="s">
         <v>12</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" s="27" t="s">
-        <v>13</v>
       </c>
       <c r="F2" s="22"/>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B3" s="34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
@@ -1122,27 +1123,27 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1150,7 +1151,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F16" s="19"/>
     </row>
@@ -1159,49 +1160,49 @@
     </row>
     <row r="18" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C18" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="G18" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="H18" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="I18" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="J18" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="K18" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="L18" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="M18" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="N18" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="O18" s="22" t="s">
         <v>28</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="E18" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="F18" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="G18" s="23" t="s">
-        <v>5</v>
-      </c>
-      <c r="H18" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="I18" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="J18" s="23" t="s">
-        <v>58</v>
-      </c>
-      <c r="K18" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="L18" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="M18" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="N18" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="O18" s="22" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1215,40 +1216,38 @@
         <v>3600</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F19" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="43" t="s">
+        <v>94</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="L19" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="K19" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L19" s="5" t="s">
-        <v>34</v>
       </c>
       <c r="M19" s="5">
         <v>507382</v>
       </c>
       <c r="N19" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="O19" s="18" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="P19" s="24"/>
     </row>
@@ -1258,18 +1257,18 @@
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
       <c r="H20" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I20" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I20" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="J20" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K20" s="5"/>
       <c r="L20" s="5"/>
@@ -1284,18 +1283,18 @@
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
       <c r="E21" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
       <c r="H21" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
@@ -1314,10 +1313,10 @@
       <c r="G22" s="5"/>
       <c r="H22" s="5"/>
       <c r="I22" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J22" s="37" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
@@ -1336,10 +1335,10 @@
       <c r="G23" s="5"/>
       <c r="H23" s="5"/>
       <c r="I23" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
@@ -1359,7 +1358,7 @@
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
       <c r="J24" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
@@ -1388,22 +1387,22 @@
     </row>
     <row r="26" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="17" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
       <c r="D26" s="11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E26" s="5"/>
       <c r="F26" s="5"/>
       <c r="G26" s="5"/>
       <c r="H26" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I26" s="5"/>
       <c r="J26" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
@@ -1421,7 +1420,7 @@
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
       <c r="H27" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
@@ -1441,7 +1440,7 @@
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
       <c r="H28" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
@@ -1461,7 +1460,7 @@
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
       <c r="H29" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
@@ -1481,7 +1480,7 @@
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
       <c r="H30" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
@@ -1528,22 +1527,22 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="37" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B37" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C37" s="6" t="s">
-        <v>17</v>
-      </c>
       <c r="D37" s="27" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E37" s="27"/>
       <c r="F37" s="27"/>
@@ -1556,7 +1555,7 @@
     </row>
     <row r="38" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B38" s="8"/>
       <c r="C38" s="3"/>
@@ -1572,7 +1571,7 @@
     </row>
     <row r="39" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B39" s="2"/>
       <c r="D39" s="5"/>
@@ -1587,7 +1586,7 @@
     </row>
     <row r="40" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="36" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B40" s="12"/>
       <c r="C40" s="13"/>
@@ -1603,7 +1602,7 @@
     </row>
     <row r="41" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B41" s="5"/>
       <c r="C41" s="5"/>
@@ -1748,26 +1747,26 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B56" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D56" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E56" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.25">
@@ -1775,10 +1774,10 @@
         <v>9600</v>
       </c>
       <c r="D57" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E57" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.25">
@@ -1786,15 +1785,15 @@
         <v>8</v>
       </c>
       <c r="D58" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D59" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.25">
@@ -1804,96 +1803,96 @@
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B68" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="76" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B76" s="38" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B77" s="39" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B78" s="39" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B79" s="40" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B80" s="41" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="81" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B81" s="41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="82" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B82" s="41" t="s">
+        <v>88</v>
+      </c>
+      <c r="C82" t="s">
         <v>90</v>
-      </c>
-      <c r="C82" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="83" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B83" s="42" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added information for Isuzu's Plant 12
git-svn-id: http://10.105.1.46/svn/CCRT/Ccrt/branches/Common3700@26818 80089e14-fa6c-c64e-badd-1f0333e23b03
</commit_message>
<xml_diff>
--- a/Source/Isuzu/Isuzu Plant Matrix.xlsx
+++ b/Source/Isuzu/Isuzu Plant Matrix.xlsx
@@ -4,19 +4,18 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="1635" yWindow="1710" windowWidth="27795" windowHeight="12465"/>
+    <workbookView xWindow="1632" yWindow="1716" windowWidth="23256" windowHeight="12468"/>
   </bookViews>
   <sheets>
     <sheet name="Charlotte" sheetId="8" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="121">
   <si>
     <t>S / N</t>
   </si>
@@ -105,9 +104,6 @@
     <t>Gryphon</t>
   </si>
   <si>
-    <t>Safty Glasses</t>
-  </si>
-  <si>
     <t>Charlotte, MI</t>
   </si>
   <si>
@@ -346,6 +342,42 @@
   </si>
   <si>
     <t>6.3.2</t>
+  </si>
+  <si>
+    <t>1(Plant 5)</t>
+  </si>
+  <si>
+    <t>2(Plant 12)</t>
+  </si>
+  <si>
+    <t>3600 Single Axle</t>
+  </si>
+  <si>
+    <t>Flash Station(Plant 5)</t>
+  </si>
+  <si>
+    <t>192.168.1.220</t>
+  </si>
+  <si>
+    <t>Safety Glasses</t>
+  </si>
+  <si>
+    <t>Plant 5: 1055 Mikesell St</t>
+  </si>
+  <si>
+    <t>Plant 12: 1023 Reynolds Rd</t>
+  </si>
+  <si>
+    <t>192.168.1.117</t>
+  </si>
+  <si>
+    <t>10.1.112.3</t>
+  </si>
+  <si>
+    <t>login: DVT_Transfer pass: Q48s^PT2</t>
+  </si>
+  <si>
+    <t>Flash/Calibration Station(Plant 12)</t>
   </si>
 </sst>
 </file>
@@ -1066,27 +1098,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P88"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P89"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
-    <col min="3" max="4" width="31.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.42578125" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="32.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.42578125" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="31.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.44140625" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="32.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.44140625" customWidth="1"/>
+    <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1111,17 +1143,17 @@
     </row>
     <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B3" s="34" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>29</v>
+        <v>114</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
       <c r="F3" s="18"/>
       <c r="G3" s="24"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="B4" s="9"/>
       <c r="C4" s="2"/>
       <c r="D4" s="5"/>
@@ -1129,23 +1161,27 @@
       <c r="F4" s="18"/>
       <c r="G4" s="24"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="7"/>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="B5" s="7" t="s">
+        <v>115</v>
+      </c>
       <c r="C5" s="5"/>
       <c r="D5" s="19"/>
       <c r="E5" s="19"/>
       <c r="F5" s="18"/>
       <c r="G5" s="24"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="7"/>
+    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="B6" s="7" t="s">
+        <v>116</v>
+      </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="18"/>
       <c r="G6" s="24"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="B7" s="24"/>
       <c r="F7" s="18"/>
       <c r="G7" s="24"/>
@@ -1162,35 +1198,35 @@
       <c r="E9" s="25"/>
       <c r="F9" s="28"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
+    <row r="12" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
+    <row r="13" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
+    <row r="14" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="F15" s="19"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>22</v>
       </c>
@@ -1228,7 +1264,7 @@
         <v>25</v>
       </c>
       <c r="J18" s="23" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K18" s="23" t="s">
         <v>6</v>
@@ -1247,8 +1283,8 @@
       </c>
     </row>
     <row r="19" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="17">
-        <v>1</v>
+      <c r="A19" s="17" t="s">
+        <v>109</v>
       </c>
       <c r="B19" s="31">
         <v>507382</v>
@@ -1257,40 +1293,40 @@
         <v>3600</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F19" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="K19" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G19" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="K19" s="5" t="s">
+      <c r="L19" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="L19" s="5" t="s">
-        <v>33</v>
       </c>
       <c r="M19" s="5">
         <v>507382</v>
       </c>
       <c r="N19" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="O19" s="18" t="s">
         <v>47</v>
-      </c>
-      <c r="O19" s="18" t="s">
-        <v>48</v>
       </c>
       <c r="P19" s="24"/>
     </row>
@@ -1300,18 +1336,18 @@
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
       <c r="H20" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K20" s="5"/>
       <c r="L20" s="5"/>
@@ -1326,18 +1362,18 @@
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
       <c r="E21" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
       <c r="H21" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
@@ -1356,10 +1392,10 @@
       <c r="G22" s="5"/>
       <c r="H22" s="5"/>
       <c r="I22" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J22" s="37" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
@@ -1368,7 +1404,7 @@
       <c r="O22" s="18"/>
       <c r="P22" s="24"/>
     </row>
-    <row r="23" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="15"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1378,10 +1414,10 @@
       <c r="G23" s="5"/>
       <c r="H23" s="5"/>
       <c r="I23" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
@@ -1390,7 +1426,7 @@
       <c r="O23" s="18"/>
       <c r="P23" s="24"/>
     </row>
-    <row r="24" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="17"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1401,7 +1437,7 @@
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
       <c r="J24" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
@@ -1410,43 +1446,61 @@
       <c r="O24" s="18"/>
       <c r="P24" s="24"/>
     </row>
-    <row r="25" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="17"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
+    <row r="25" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="B25" s="5">
+        <v>508702</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>47</v>
+      </c>
       <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
-      <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
+      <c r="H25" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="J25" s="37" t="s">
+        <v>119</v>
+      </c>
+      <c r="K25" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="M25" s="5">
+        <v>508702</v>
+      </c>
       <c r="N25" s="5"/>
-      <c r="O25" s="18"/>
+      <c r="O25" s="18" t="s">
+        <v>113</v>
+      </c>
       <c r="P25" s="24"/>
     </row>
-    <row r="26" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="17" t="s">
-        <v>34</v>
-      </c>
+    <row r="26" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="17"/>
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
-      <c r="D26" s="11" t="s">
-        <v>46</v>
-      </c>
+      <c r="D26" s="11"/>
       <c r="E26" s="5"/>
       <c r="F26" s="5"/>
       <c r="G26" s="5"/>
-      <c r="H26" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="H26" s="5"/>
       <c r="I26" s="5"/>
-      <c r="J26" s="5" t="s">
-        <v>60</v>
-      </c>
+      <c r="J26" s="5"/>
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
       <c r="M26" s="5"/>
@@ -1454,19 +1508,25 @@
       <c r="O26" s="18"/>
       <c r="P26" s="24"/>
     </row>
-    <row r="27" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="17"/>
+    <row r="27" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="17" t="s">
+        <v>112</v>
+      </c>
       <c r="B27" s="11"/>
       <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
+      <c r="D27" s="11" t="s">
+        <v>45</v>
+      </c>
       <c r="E27" s="5"/>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
       <c r="H27" s="5" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
+      <c r="J27" s="5" t="s">
+        <v>59</v>
+      </c>
       <c r="K27" s="5"/>
       <c r="L27" s="5"/>
       <c r="M27" s="5"/>
@@ -1474,8 +1534,8 @@
       <c r="O27" s="18"/>
       <c r="P27" s="24"/>
     </row>
-    <row r="28" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="14"/>
+    <row r="28" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="17"/>
       <c r="B28" s="11"/>
       <c r="C28" s="11"/>
       <c r="D28" s="11"/>
@@ -1483,7 +1543,7 @@
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
       <c r="H28" s="5" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
@@ -1494,7 +1554,7 @@
       <c r="O28" s="18"/>
       <c r="P28" s="24"/>
     </row>
-    <row r="29" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="14"/>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -1503,7 +1563,7 @@
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
       <c r="H29" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
@@ -1514,8 +1574,8 @@
       <c r="O29" s="18"/>
       <c r="P29" s="24"/>
     </row>
-    <row r="30" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="16"/>
+    <row r="30" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="14"/>
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
       <c r="D30" s="11"/>
@@ -1523,7 +1583,7 @@
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
       <c r="H30" s="5" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
@@ -1534,15 +1594,17 @@
       <c r="O30" s="18"/>
       <c r="P30" s="24"/>
     </row>
-    <row r="31" spans="1:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="15"/>
-      <c r="B31" s="32"/>
-      <c r="C31" s="32"/>
+    <row r="31" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="16"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
       <c r="D31" s="11"/>
       <c r="E31" s="5"/>
       <c r="F31" s="5"/>
       <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
+      <c r="H31" s="5" t="s">
+        <v>65</v>
+      </c>
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
       <c r="K31" s="5"/>
@@ -1552,90 +1614,96 @@
       <c r="O31" s="18"/>
       <c r="P31" s="24"/>
     </row>
-    <row r="32" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="25"/>
-      <c r="C32" s="25"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="25"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="25"/>
-      <c r="H32" s="25"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="28"/>
-      <c r="K32" s="25"/>
-      <c r="L32" s="25"/>
-      <c r="M32" s="28"/>
-      <c r="N32" s="25"/>
-      <c r="O32" s="25"/>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A35" s="10" t="s">
+    <row r="32" spans="1:16" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="5"/>
+      <c r="L32" s="5"/>
+      <c r="M32" s="5"/>
+      <c r="N32" s="5"/>
+      <c r="O32" s="18"/>
+      <c r="P32" s="24"/>
+    </row>
+    <row r="33" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="25"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="25"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="28"/>
+      <c r="K33" s="25"/>
+      <c r="L33" s="25"/>
+      <c r="M33" s="28"/>
+      <c r="N33" s="25"/>
+      <c r="O33" s="25"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A36" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="37" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
+    <row r="37" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="38" spans="1:15" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B38" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C38" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D37" s="27" t="s">
+      <c r="D38" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="E37" s="27"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="27"/>
-      <c r="I37" s="27"/>
-      <c r="J37" s="27"/>
-      <c r="K37" s="22"/>
-      <c r="L37" s="21"/>
-    </row>
-    <row r="38" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="17" t="s">
+      <c r="E38" s="27"/>
+      <c r="F38" s="27"/>
+      <c r="G38" s="27"/>
+      <c r="H38" s="27"/>
+      <c r="I38" s="27"/>
+      <c r="J38" s="27"/>
+      <c r="K38" s="22"/>
+      <c r="L38" s="21"/>
+    </row>
+    <row r="39" spans="1:15" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="8"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
-      <c r="K38" s="28"/>
-      <c r="L38" s="24"/>
-    </row>
-    <row r="39" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="36" t="s">
+      <c r="B39" s="8"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="2"/>
+      <c r="K39" s="28"/>
+      <c r="L39" s="24"/>
+    </row>
+    <row r="40" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="B39" s="2"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="19"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="19"/>
-      <c r="J39" s="19"/>
-      <c r="K39" s="18"/>
-      <c r="L39" s="24"/>
-    </row>
-    <row r="40" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="36" t="s">
-        <v>18</v>
-      </c>
-      <c r="B40" s="12"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="29"/>
-      <c r="E40" s="30"/>
-      <c r="F40" s="30"/>
+      <c r="B40" s="2"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
       <c r="G40" s="19"/>
       <c r="H40" s="19"/>
       <c r="I40" s="19"/>
@@ -1643,15 +1711,15 @@
       <c r="K40" s="18"/>
       <c r="L40" s="24"/>
     </row>
-    <row r="41" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="B41" s="5"/>
-      <c r="C41" s="5"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="19"/>
+    <row r="41" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="B41" s="12"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="30"/>
+      <c r="F41" s="30"/>
       <c r="G41" s="19"/>
       <c r="H41" s="19"/>
       <c r="I41" s="19"/>
@@ -1659,12 +1727,14 @@
       <c r="K41" s="18"/>
       <c r="L41" s="24"/>
     </row>
-    <row r="42" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="16"/>
+    <row r="42" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="16" t="s">
+        <v>12</v>
+      </c>
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
-      <c r="D42" s="19"/>
-      <c r="E42" s="19"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
       <c r="F42" s="19"/>
       <c r="G42" s="19"/>
       <c r="H42" s="19"/>
@@ -1673,9 +1743,10 @@
       <c r="K42" s="18"/>
       <c r="L42" s="24"/>
     </row>
-    <row r="43" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="15"/>
-      <c r="B43" s="2"/>
+    <row r="43" spans="1:15" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="16"/>
+      <c r="B43" s="5"/>
+      <c r="C43" s="5"/>
       <c r="D43" s="19"/>
       <c r="E43" s="19"/>
       <c r="F43" s="19"/>
@@ -1686,7 +1757,7 @@
       <c r="K43" s="18"/>
       <c r="L43" s="24"/>
     </row>
-    <row r="44" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:15" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="15"/>
       <c r="B44" s="2"/>
       <c r="D44" s="19"/>
@@ -1699,7 +1770,7 @@
       <c r="K44" s="18"/>
       <c r="L44" s="24"/>
     </row>
-    <row r="45" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:15" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="15"/>
       <c r="B45" s="2"/>
       <c r="D45" s="19"/>
@@ -1712,7 +1783,7 @@
       <c r="K45" s="18"/>
       <c r="L45" s="24"/>
     </row>
-    <row r="46" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:15" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="15"/>
       <c r="B46" s="2"/>
       <c r="D46" s="19"/>
@@ -1725,7 +1796,7 @@
       <c r="K46" s="18"/>
       <c r="L46" s="24"/>
     </row>
-    <row r="47" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:15" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="15"/>
       <c r="B47" s="2"/>
       <c r="D47" s="19"/>
@@ -1738,7 +1809,7 @@
       <c r="K47" s="18"/>
       <c r="L47" s="24"/>
     </row>
-    <row r="48" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:15" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="15"/>
       <c r="B48" s="2"/>
       <c r="D48" s="19"/>
@@ -1751,7 +1822,7 @@
       <c r="K48" s="18"/>
       <c r="L48" s="24"/>
     </row>
-    <row r="49" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="15"/>
       <c r="B49" s="2"/>
       <c r="D49" s="19"/>
@@ -1764,231 +1835,244 @@
       <c r="K49" s="18"/>
       <c r="L49" s="24"/>
     </row>
-    <row r="50" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="15"/>
-      <c r="B50" s="4"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-      <c r="G50" s="2"/>
-      <c r="H50" s="2"/>
-      <c r="I50" s="2"/>
-      <c r="J50" s="2"/>
-      <c r="K50" s="33"/>
+      <c r="B50" s="2"/>
+      <c r="D50" s="19"/>
+      <c r="E50" s="19"/>
+      <c r="F50" s="19"/>
+      <c r="G50" s="19"/>
+      <c r="H50" s="19"/>
+      <c r="I50" s="19"/>
+      <c r="J50" s="19"/>
+      <c r="K50" s="18"/>
       <c r="L50" s="24"/>
     </row>
-    <row r="51" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="D51" s="25"/>
-      <c r="E51" s="25"/>
-      <c r="F51" s="28"/>
-      <c r="G51" s="25"/>
-      <c r="H51" s="25"/>
-      <c r="I51" s="28"/>
-      <c r="J51" s="28"/>
-      <c r="K51" s="25"/>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A54" s="10" t="s">
+    <row r="51" spans="1:12" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="15"/>
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="2"/>
+      <c r="K51" s="33"/>
+      <c r="L51" s="24"/>
+    </row>
+    <row r="52" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="D52" s="25"/>
+      <c r="E52" s="25"/>
+      <c r="F52" s="28"/>
+      <c r="G52" s="25"/>
+      <c r="H52" s="25"/>
+      <c r="I52" s="28"/>
+      <c r="J52" s="28"/>
+      <c r="K52" s="25"/>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A55" s="10" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>33</v>
+      </c>
+      <c r="B57" t="s">
         <v>34</v>
       </c>
-      <c r="B56" t="s">
-        <v>35</v>
-      </c>
-      <c r="D56" t="s">
-        <v>38</v>
-      </c>
-      <c r="E56" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B57">
+      <c r="D57" t="s">
+        <v>37</v>
+      </c>
+      <c r="E57" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B58">
         <v>9600</v>
-      </c>
-      <c r="D57" t="s">
-        <v>40</v>
-      </c>
-      <c r="E57" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B58">
-        <v>8</v>
       </c>
       <c r="D58" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B59" t="s">
+      <c r="E58" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B59">
+        <v>8</v>
+      </c>
+      <c r="D59" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B60" t="s">
+        <v>35</v>
+      </c>
+      <c r="D60" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B62" t="s">
         <v>36</v>
       </c>
-      <c r="D59" t="s">
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B64" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B65" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B60">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B61" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B63" t="s">
+      <c r="B69" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B70" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B64" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>42</v>
-      </c>
-      <c r="B68" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B69" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+      <c r="D74" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D75" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D76" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
         <v>78</v>
       </c>
-      <c r="D73" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D74" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D75" t="s">
+      <c r="B77" s="38" t="s">
+        <v>82</v>
+      </c>
+      <c r="D77" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
+    <row r="78" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>79</v>
       </c>
-      <c r="B76" s="38" t="s">
+      <c r="B78" s="39" t="s">
         <v>83</v>
       </c>
-      <c r="D76" t="s">
+      <c r="D78" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
+    <row r="79" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
         <v>80</v>
       </c>
-      <c r="B77" s="39" t="s">
+      <c r="B79" s="39" t="s">
         <v>84</v>
       </c>
-      <c r="D77" t="s">
+      <c r="D79" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
+    <row r="80" spans="1:4" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
         <v>81</v>
       </c>
-      <c r="B78" s="39" t="s">
+      <c r="B80" s="40" t="s">
         <v>85</v>
       </c>
-      <c r="D78" t="s">
+      <c r="D80" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="79" spans="1:4" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>82</v>
-      </c>
-      <c r="B79" s="40" t="s">
+    <row r="81" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B81" s="41" t="s">
         <v>86</v>
       </c>
-      <c r="D79" t="s">
+      <c r="D81" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B80" s="41" t="s">
+    <row r="82" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B82" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="D80" t="s">
+    </row>
+    <row r="83" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B83" s="41" t="s">
+        <v>88</v>
+      </c>
+      <c r="C83" t="s">
+        <v>90</v>
+      </c>
+      <c r="D83" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="81" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B81" s="41" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="82" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B82" s="41" t="s">
+    <row r="84" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B84" s="42" t="s">
         <v>89</v>
       </c>
-      <c r="C82" t="s">
-        <v>91</v>
-      </c>
-      <c r="D82" t="s">
+      <c r="D84" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="83" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="42" t="s">
-        <v>90</v>
-      </c>
-      <c r="D83" t="s">
+    <row r="85" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D85" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="84" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D84" t="s">
+    <row r="87" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D87" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="86" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D86" t="s">
+    <row r="88" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D88" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="87" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D87" t="s">
+    <row r="89" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="D89" t="s">
         <v>107</v>
-      </c>
-    </row>
-    <row r="88" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D88" t="s">
-        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2000,16 +2084,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>